<commit_message>
fix(seguimiento): update excel template and enforce strict undefined for empty cells to fix formulas
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0156GGX9ZEFQzauogTkjrDYT
</commit_message>
<xml_diff>
--- a/assets/docs/Seguimiento_de_Carrera.xlsx
+++ b/assets/docs/Seguimiento_de_Carrera.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://frreutn-my.sharepoint.com/personal/lautyyzalazar2_ca_frre_utn_edu_ar/Documents/UTN/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{97B535F0-D1C1-49FE-ADEB-99B00EA5739A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="74" documentId="8_{97B535F0-D1C1-49FE-ADEB-99B00EA5739A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EDE4952C-874F-456D-8FC0-7B2CA63050A5}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{3EE8B6AE-4571-404E-BC87-750763CF3DE4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{3EE8B6AE-4571-404E-BC87-750763CF3DE4}"/>
   </bookViews>
   <sheets>
     <sheet name="Seguimiento" sheetId="1" r:id="rId1"/>
@@ -2339,24 +2339,144 @@
     <xf numFmtId="0" fontId="9" fillId="13" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="29" fillId="5" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="5" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="5" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="31" fillId="6" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="6" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="35" fillId="11" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="12" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="37" fillId="12" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="11" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="12" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="37" fillId="12" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="12" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="29" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="29" fillId="5" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="31" fillId="6" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="11" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="12" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="40" fillId="11" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="12" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="43" fillId="10" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="10" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="45" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="44" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="10" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="10" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="43" fillId="10" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -2365,132 +2485,144 @@
     </xf>
     <xf numFmtId="0" fontId="43" fillId="10" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="29" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="29" fillId="5" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="31" fillId="6" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="11" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="12" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="40" fillId="11" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="12" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="29" fillId="5" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="5" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="31" fillId="6" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="6" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="35" fillId="11" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="12" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="37" fillId="12" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="11" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="12" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="37" fillId="12" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="12" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="27">
+  <dxfs count="39">
+    <dxf>
+      <font>
+        <color rgb="FF991B1B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF065F46"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFD1FAE5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF991B1B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF065F46"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFD1FAE5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF991B1B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF065F46"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFD1FAE5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF991B1B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF065F46"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFD1FAE5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF991B1B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF065F46"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFD1FAE5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF991B1B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF065F46"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFD1FAE5"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF991B1B"/>
@@ -3402,10 +3534,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
@@ -3761,17 +3889,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="270" t="s">
+      <c r="A1" s="250" t="s">
         <v>124</v>
       </c>
-      <c r="B1" s="270"/>
-      <c r="C1" s="270"/>
-      <c r="D1" s="270"/>
-      <c r="E1" s="270"/>
-      <c r="F1" s="270"/>
-      <c r="G1" s="270"/>
-      <c r="H1" s="270"/>
-      <c r="I1" s="270"/>
+      <c r="B1" s="250"/>
+      <c r="C1" s="250"/>
+      <c r="D1" s="250"/>
+      <c r="E1" s="250"/>
+      <c r="F1" s="250"/>
+      <c r="G1" s="250"/>
+      <c r="H1" s="250"/>
+      <c r="I1" s="250"/>
       <c r="J1" s="7"/>
       <c r="K1" s="4"/>
       <c r="L1" s="2"/>
@@ -3792,17 +3920,17 @@
       <c r="AA1" s="2"/>
     </row>
     <row r="2" spans="1:27" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="271" t="s">
+      <c r="A2" s="251" t="s">
         <v>125</v>
       </c>
-      <c r="B2" s="271"/>
-      <c r="C2" s="271"/>
-      <c r="D2" s="271"/>
-      <c r="E2" s="271"/>
-      <c r="F2" s="271"/>
-      <c r="G2" s="271"/>
-      <c r="H2" s="271"/>
-      <c r="I2" s="271"/>
+      <c r="B2" s="251"/>
+      <c r="C2" s="251"/>
+      <c r="D2" s="251"/>
+      <c r="E2" s="251"/>
+      <c r="F2" s="251"/>
+      <c r="G2" s="251"/>
+      <c r="H2" s="251"/>
+      <c r="I2" s="251"/>
       <c r="J2" s="8"/>
       <c r="K2" s="4"/>
       <c r="L2" s="2"/>
@@ -3852,26 +3980,26 @@
       <c r="AA3" s="2"/>
     </row>
     <row r="4" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="274" t="s">
+      <c r="A4" s="254" t="s">
         <v>126</v>
       </c>
-      <c r="B4" s="274"/>
-      <c r="C4" s="277" t="s">
+      <c r="B4" s="254"/>
+      <c r="C4" s="257" t="s">
         <v>128</v>
       </c>
-      <c r="D4" s="274"/>
-      <c r="E4" s="280" t="s">
+      <c r="D4" s="254"/>
+      <c r="E4" s="260" t="s">
         <v>165</v>
       </c>
-      <c r="F4" s="281"/>
-      <c r="G4" s="284" t="s">
+      <c r="F4" s="261"/>
+      <c r="G4" s="264" t="s">
         <v>143</v>
       </c>
-      <c r="H4" s="285"/>
-      <c r="I4" s="288" t="s">
+      <c r="H4" s="265"/>
+      <c r="I4" s="268" t="s">
         <v>167</v>
       </c>
-      <c r="J4" s="289"/>
+      <c r="J4" s="269"/>
       <c r="K4" s="4"/>
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
@@ -3891,31 +4019,31 @@
       <c r="AA4" s="2"/>
     </row>
     <row r="5" spans="1:27" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="275">
+      <c r="A5" s="255">
         <f>COUNTIF(F12:F64,"Aprobada")</f>
         <v>0</v>
       </c>
-      <c r="B5" s="276"/>
-      <c r="C5" s="278">
+      <c r="B5" s="256"/>
+      <c r="C5" s="258">
         <f>IFERROR(COUNTIF(F12:F52,"Aprobada")/41,0)</f>
         <v>0</v>
       </c>
-      <c r="D5" s="279"/>
-      <c r="E5" s="282">
+      <c r="D5" s="259"/>
+      <c r="E5" s="262">
         <f>COUNTIF(F12:F52,"No Cursada")+COUNTIF(F12:F52,"Cursando")</f>
         <v>41</v>
       </c>
-      <c r="F5" s="283"/>
-      <c r="G5" s="286" t="str">
+      <c r="F5" s="263"/>
+      <c r="G5" s="266" t="str">
         <f>IFERROR(AVERAGEIF(G12:G64,"&gt;="&amp;6),"—")</f>
         <v>—</v>
       </c>
-      <c r="H5" s="287"/>
-      <c r="I5" s="290" cm="1">
+      <c r="H5" s="267"/>
+      <c r="I5" s="270" cm="1">
         <f t="array" ref="I5">SUMPRODUCT((F53:F65="Aprobada")*J53:J65)</f>
         <v>0</v>
       </c>
-      <c r="J5" s="291"/>
+      <c r="J5" s="271"/>
       <c r="K5" s="4"/>
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
@@ -3935,24 +4063,24 @@
       <c r="AA5" s="2"/>
     </row>
     <row r="6" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="296" t="s">
+      <c r="A6" s="276" t="s">
         <v>166</v>
       </c>
-      <c r="B6" s="296"/>
-      <c r="C6" s="296"/>
-      <c r="D6" s="297"/>
-      <c r="E6" s="263" t="s">
+      <c r="B6" s="276"/>
+      <c r="C6" s="276"/>
+      <c r="D6" s="277"/>
+      <c r="E6" s="280" t="s">
         <v>127</v>
       </c>
-      <c r="F6" s="263"/>
-      <c r="G6" s="266" t="s">
+      <c r="F6" s="280"/>
+      <c r="G6" s="283" t="s">
         <v>144</v>
       </c>
-      <c r="H6" s="267"/>
-      <c r="I6" s="292" t="s">
+      <c r="H6" s="284"/>
+      <c r="I6" s="272" t="s">
         <v>168</v>
       </c>
-      <c r="J6" s="293"/>
+      <c r="J6" s="273"/>
       <c r="K6" s="4"/>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
@@ -3972,28 +4100,28 @@
       <c r="AA6" s="2"/>
     </row>
     <row r="7" spans="1:27" ht="44.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="261">
+      <c r="A7" s="278">
         <f>COUNTIF(H12:H52,"✅ Disponible")</f>
         <v>9</v>
       </c>
-      <c r="B7" s="261"/>
-      <c r="C7" s="261"/>
-      <c r="D7" s="262"/>
-      <c r="E7" s="264">
+      <c r="B7" s="278"/>
+      <c r="C7" s="278"/>
+      <c r="D7" s="279"/>
+      <c r="E7" s="281">
         <f>COUNTIF(F12:F64,"Regular")</f>
         <v>0</v>
       </c>
-      <c r="F7" s="265"/>
-      <c r="G7" s="268" t="str" cm="1">
+      <c r="F7" s="282"/>
+      <c r="G7" s="285" t="str" cm="1">
         <f t="array" ref="G7">IFERROR((SUMPRODUCT(IF(ISNUMBER(G12:G64),G12:G64,0))+SUMPRODUCT((ISNUMBER(Finales!G5:G57))*(Finales!G5:G57&lt;6)*Finales!G5:G57)+SUMPRODUCT((ISNUMBER(Finales!I5:I57))*(Finales!I5:I57&lt;6)*Finales!I5:I57)+SUMPRODUCT((ISNUMBER(Finales!K5:K57))*(Finales!K5:K57&lt;6)*Finales!K5:K57)+SUMPRODUCT((ISNUMBER(Finales!M5:M57))*(Finales!M5:M57&lt;6)*Finales!M5:M57)+SUMPRODUCT((ISNUMBER(Finales!O5:O57))*(Finales!O5:O57&lt;6)*Finales!O5:O57)+SUMPRODUCT((ISNUMBER(Finales!Q5:Q57))*(Finales!Q5:Q57&lt;6)*Finales!Q5:Q57))/(SUMPRODUCT(ISNUMBER(G12:G64)*1)+SUMPRODUCT((ISNUMBER(Finales!G5:G57))*(Finales!G5:G57&lt;6))+SUMPRODUCT((ISNUMBER(Finales!I5:I57))*(Finales!I5:I57&lt;6))+SUMPRODUCT((ISNUMBER(Finales!K5:K57))*(Finales!K5:K57&lt;6))+SUMPRODUCT((ISNUMBER(Finales!M5:M57))*(Finales!M5:M57&lt;6))+SUMPRODUCT((ISNUMBER(Finales!O5:O57))*(Finales!O5:O57&lt;6))+SUMPRODUCT((ISNUMBER(Finales!Q5:Q57))*(Finales!Q5:Q57&lt;6))),"—")</f>
         <v>—</v>
       </c>
-      <c r="H7" s="269"/>
-      <c r="I7" s="294" cm="1">
+      <c r="H7" s="286"/>
+      <c r="I7" s="274" cm="1">
         <f t="array" ref="I7">IFERROR(SUMPRODUCT((F53:F65="Aprobada")*J53:J65)/24,0)</f>
         <v>0</v>
       </c>
-      <c r="J7" s="295"/>
+      <c r="J7" s="275"/>
       <c r="K7" s="4"/>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
@@ -4013,17 +4141,17 @@
       <c r="AA7" s="2"/>
     </row>
     <row r="8" spans="1:27" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="272" t="s">
+      <c r="A8" s="252" t="s">
         <v>147</v>
       </c>
-      <c r="B8" s="273"/>
-      <c r="C8" s="273"/>
-      <c r="D8" s="273"/>
-      <c r="E8" s="273"/>
-      <c r="F8" s="273"/>
-      <c r="G8" s="273"/>
-      <c r="H8" s="273"/>
-      <c r="I8" s="273"/>
+      <c r="B8" s="253"/>
+      <c r="C8" s="253"/>
+      <c r="D8" s="253"/>
+      <c r="E8" s="253"/>
+      <c r="F8" s="253"/>
+      <c r="G8" s="253"/>
+      <c r="H8" s="253"/>
+      <c r="I8" s="253"/>
       <c r="J8" s="9"/>
       <c r="K8" s="4"/>
       <c r="L8" s="2"/>
@@ -8005,6 +8133,11 @@
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="21">
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="G7:H7"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A8:I8"/>
@@ -8021,54 +8154,49 @@
     <mergeCell ref="I6:J6"/>
     <mergeCell ref="I7:J7"/>
     <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="G7:H7"/>
   </mergeCells>
   <conditionalFormatting sqref="F12:F65">
-    <cfRule type="containsText" dxfId="26" priority="17" operator="containsText" text="Aprobada">
+    <cfRule type="containsText" dxfId="38" priority="17" operator="containsText" text="Aprobada">
       <formula>NOT(ISERROR(SEARCH("Aprobada",F12)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="25" priority="18" operator="containsText" text="Regular">
+    <cfRule type="containsText" dxfId="37" priority="18" operator="containsText" text="Regular">
       <formula>NOT(ISERROR(SEARCH("Regular",F12)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="24" priority="19" operator="containsText" text="Cursando">
+    <cfRule type="containsText" dxfId="36" priority="19" operator="containsText" text="Cursando">
       <formula>NOT(ISERROR(SEARCH("Cursando",F12)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="23" priority="20" operator="containsText" text="No Cursada">
+    <cfRule type="containsText" dxfId="35" priority="20" operator="containsText" text="No Cursada">
       <formula>NOT(ISERROR(SEARCH("No Cursada",F12)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G12:G65">
-    <cfRule type="containsText" dxfId="22" priority="13" operator="containsText" text="Aprobada">
+    <cfRule type="containsText" dxfId="34" priority="13" operator="containsText" text="Aprobada">
       <formula>NOT(ISERROR(SEARCH("Aprobada",G12)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="21" priority="14" operator="containsText" text="Regular">
+    <cfRule type="containsText" dxfId="33" priority="14" operator="containsText" text="Regular">
       <formula>NOT(ISERROR(SEARCH("Regular",G12)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="20" priority="15" operator="containsText" text="Cursando">
+    <cfRule type="containsText" dxfId="32" priority="15" operator="containsText" text="Cursando">
       <formula>NOT(ISERROR(SEARCH("Cursando",G12)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="19" priority="16" operator="containsText" text="No Cursada">
+    <cfRule type="containsText" dxfId="31" priority="16" operator="containsText" text="No Cursada">
       <formula>NOT(ISERROR(SEARCH("No Cursada",G12)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12:H52">
-    <cfRule type="containsText" dxfId="18" priority="4" operator="containsText" text="Disponible">
+    <cfRule type="containsText" dxfId="30" priority="4" operator="containsText" text="Disponible">
       <formula>NOT(ISERROR(SEARCH("Disponible",H12)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="17" priority="5" operator="containsText" text="Aprobada">
+    <cfRule type="containsText" dxfId="29" priority="5" operator="containsText" text="Aprobada">
       <formula>NOT(ISERROR(SEARCH("Aprobada",H12)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="16" priority="6" operator="containsText" text="Regular">
+    <cfRule type="containsText" dxfId="28" priority="6" operator="containsText" text="Regular">
       <formula>NOT(ISERROR(SEARCH("Regular",H12)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="15" priority="7" operator="containsText" text="No Disponible">
+    <cfRule type="containsText" dxfId="27" priority="7" operator="containsText" text="No Disponible">
       <formula>NOT(ISERROR(SEARCH("No Disponible",H12)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="12" operator="containsText" text="Cursando">
+    <cfRule type="containsText" dxfId="26" priority="12" operator="containsText" text="Cursando">
       <formula>NOT(ISERROR(SEARCH("Cursando",H12)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8111,42 +8239,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="270" t="s">
+      <c r="A1" s="250" t="s">
         <v>137</v>
       </c>
-      <c r="B1" s="270"/>
-      <c r="C1" s="270"/>
-      <c r="D1" s="270"/>
-      <c r="E1" s="270"/>
-      <c r="F1" s="270"/>
-      <c r="G1" s="270"/>
-      <c r="H1" s="270"/>
-      <c r="I1" s="270"/>
-      <c r="J1" s="270"/>
-      <c r="K1" s="270"/>
-      <c r="L1" s="270"/>
-      <c r="M1" s="270"/>
+      <c r="B1" s="250"/>
+      <c r="C1" s="250"/>
+      <c r="D1" s="250"/>
+      <c r="E1" s="250"/>
+      <c r="F1" s="250"/>
+      <c r="G1" s="250"/>
+      <c r="H1" s="250"/>
+      <c r="I1" s="250"/>
+      <c r="J1" s="250"/>
+      <c r="K1" s="250"/>
+      <c r="L1" s="250"/>
+      <c r="M1" s="250"/>
       <c r="N1" s="7"/>
       <c r="O1" s="7"/>
       <c r="P1" s="7"/>
       <c r="Q1" s="7"/>
     </row>
     <row r="2" spans="1:17" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="298" t="s">
+      <c r="A2" s="287" t="s">
         <v>138</v>
       </c>
-      <c r="B2" s="298"/>
-      <c r="C2" s="298"/>
-      <c r="D2" s="298"/>
-      <c r="E2" s="298"/>
-      <c r="F2" s="298"/>
-      <c r="G2" s="298"/>
-      <c r="H2" s="298"/>
-      <c r="I2" s="298"/>
-      <c r="J2" s="298"/>
-      <c r="K2" s="298"/>
-      <c r="L2" s="298"/>
-      <c r="M2" s="298"/>
+      <c r="B2" s="287"/>
+      <c r="C2" s="287"/>
+      <c r="D2" s="287"/>
+      <c r="E2" s="287"/>
+      <c r="F2" s="287"/>
+      <c r="G2" s="287"/>
+      <c r="H2" s="287"/>
+      <c r="I2" s="287"/>
+      <c r="J2" s="287"/>
+      <c r="K2" s="287"/>
+      <c r="L2" s="287"/>
+      <c r="M2" s="287"/>
       <c r="N2" s="38"/>
       <c r="O2" s="38"/>
       <c r="P2" s="38"/>
@@ -9905,64 +10033,141 @@
     <mergeCell ref="A2:M2"/>
   </mergeCells>
   <conditionalFormatting sqref="D5:D45">
-    <cfRule type="containsText" dxfId="13" priority="9" operator="containsText" text="Aprobada">
+    <cfRule type="containsText" dxfId="25" priority="9" operator="containsText" text="Aprobada">
       <formula>NOT(ISERROR(SEARCH("Aprobada",D5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="12" priority="10" operator="containsText" text="Regular">
+    <cfRule type="containsText" dxfId="24" priority="10" operator="containsText" text="Regular">
       <formula>NOT(ISERROR(SEARCH("Regular",D5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="11" priority="11" operator="containsText" text="Cursando">
+    <cfRule type="containsText" dxfId="23" priority="11" operator="containsText" text="Cursando">
       <formula>NOT(ISERROR(SEARCH("Cursando",D5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="12" operator="containsText" text="No Cursada">
+    <cfRule type="containsText" dxfId="22" priority="12" operator="containsText" text="No Cursada">
       <formula>NOT(ISERROR(SEARCH("No Cursada",D5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D5:D58">
-    <cfRule type="containsText" dxfId="9" priority="13" operator="containsText" text="No Cursada">
+    <cfRule type="containsText" dxfId="21" priority="13" operator="containsText" text="No Cursada">
       <formula>NOT(ISERROR(SEARCH("No Cursada",D5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="14" operator="containsText" text="Cursando">
+    <cfRule type="containsText" dxfId="20" priority="14" operator="containsText" text="Cursando">
       <formula>NOT(ISERROR(SEARCH("Cursando",D5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="7" priority="15" operator="containsText" text="Regular">
+    <cfRule type="containsText" dxfId="19" priority="15" operator="containsText" text="Regular">
       <formula>NOT(ISERROR(SEARCH("Regular",D5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="16" operator="containsText" text="Aprobada">
+    <cfRule type="containsText" dxfId="18" priority="16" operator="containsText" text="Aprobada">
       <formula>NOT(ISERROR(SEARCH("Aprobada",D5)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H5:H45">
-    <cfRule type="cellIs" dxfId="5" priority="3" operator="greaterThanOrEqual">
+  <conditionalFormatting sqref="G5:G58">
+    <cfRule type="cellIs" dxfId="11" priority="17" operator="greaterThanOrEqual">
       <formula>6</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="4" operator="between">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G5:G58">
+    <cfRule type="cellIs" dxfId="10" priority="18" operator="between">
       <formula>1</formula>
       <formula>5</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J5:J45">
-    <cfRule type="cellIs" dxfId="3" priority="5" operator="greaterThanOrEqual">
+  <conditionalFormatting sqref="I5:I58">
+    <cfRule type="cellIs" dxfId="9" priority="19" operator="greaterThanOrEqual">
       <formula>6</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="6" operator="between">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I5:I58">
+    <cfRule type="cellIs" dxfId="8" priority="20" operator="between">
       <formula>1</formula>
       <formula>5</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L5:L45">
-    <cfRule type="cellIs" dxfId="1" priority="7" operator="greaterThanOrEqual">
+  <conditionalFormatting sqref="K5:K58">
+    <cfRule type="cellIs" dxfId="7" priority="21" operator="greaterThanOrEqual">
       <formula>6</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="8" operator="between">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K5:K58">
+    <cfRule type="cellIs" dxfId="6" priority="22" operator="between">
       <formula>1</formula>
       <formula>5</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Nota inválida" error="La nota debe ser un número entre 1 y 10." promptTitle="Nota de Final" prompt="Ingrese la nota del examen final (1-10). Se aprueba con 6." sqref="H5:H45 L5:L45 J5:J45" xr:uid="{147E68F6-8A30-46C0-A4F8-512EEDA1E16E}">
+  <conditionalFormatting sqref="M5:M58">
+    <cfRule type="cellIs" dxfId="5" priority="23" operator="greaterThanOrEqual">
+      <formula>6</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M5:M58">
+    <cfRule type="cellIs" dxfId="4" priority="24" operator="between">
+      <formula>1</formula>
+      <formula>5</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O5:O58">
+    <cfRule type="cellIs" dxfId="3" priority="25" operator="greaterThanOrEqual">
+      <formula>6</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O5:O58">
+    <cfRule type="cellIs" dxfId="2" priority="26" operator="between">
+      <formula>1</formula>
+      <formula>5</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q5:Q58">
+    <cfRule type="cellIs" dxfId="1" priority="27" operator="greaterThanOrEqual">
+      <formula>6</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q5:Q58">
+    <cfRule type="cellIs" dxfId="0" priority="28" operator="between">
+      <formula>1</formula>
+      <formula>5</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="12">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Nota invalida" error="La nota debe ser un numero entero entre 1 y 10." sqref="G5:G58" xr:uid="{EF5A2524-3694-4256-A2FB-6636E3EE64E6}">
       <formula1>1</formula1>
       <formula2>10</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Nota invalida" error="La nota debe ser un numero entero entre 1 y 10." sqref="I5:I58" xr:uid="{CF6791EF-E203-433B-91E7-CE121B324BAA}">
+      <formula1>1</formula1>
+      <formula2>10</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Nota invalida" error="La nota debe ser un numero entero entre 1 y 10." sqref="K5:K58" xr:uid="{E1F3E34A-DA5C-4678-8B58-52AE3552A556}">
+      <formula1>1</formula1>
+      <formula2>10</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Nota invalida" error="La nota debe ser un numero entero entre 1 y 10." sqref="M5:M58" xr:uid="{E12FE5DB-6F1B-478D-B91C-0DEDB4706089}">
+      <formula1>1</formula1>
+      <formula2>10</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Nota invalida" error="La nota debe ser un numero entero entre 1 y 10." sqref="O5:O58" xr:uid="{88C66DD0-DF81-4DA2-9D48-373B49305FBA}">
+      <formula1>1</formula1>
+      <formula2>10</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Nota invalida" error="La nota debe ser un numero entero entre 1 y 10." sqref="Q5:Q58" xr:uid="{1E5F17FF-8E08-4F81-9529-5D1EB9733CEE}">
+      <formula1>1</formula1>
+      <formula2>10</formula2>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Fecha invalida" error="Ingrese una fecha valida (por ejemplo 15/03/2025)." sqref="F5:F58" xr:uid="{2FCD9CF0-27B5-4E3C-A02F-0A0FCA30BAB0}">
+      <formula1>AND(ISNUMBER(F5),F5&gt;=36526)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Fecha invalida" error="Ingrese una fecha valida (por ejemplo 15/03/2025)." sqref="H5:H58" xr:uid="{9B8CB559-180F-424E-99BB-1B2D9E090B2F}">
+      <formula1>AND(ISNUMBER(H5),H5&gt;=36526)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Fecha invalida" error="Ingrese una fecha valida (por ejemplo 15/03/2025)." sqref="J5:J58" xr:uid="{6B87AF2E-2704-4F97-9A3D-00F036C07877}">
+      <formula1>AND(ISNUMBER(J5),J5&gt;=36526)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Fecha invalida" error="Ingrese una fecha valida (por ejemplo 15/03/2025)." sqref="L5:L58" xr:uid="{747FE15A-A324-46A4-88C6-73F51E7BD81C}">
+      <formula1>AND(ISNUMBER(L5),L5&gt;=36526)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Fecha invalida" error="Ingrese una fecha valida (por ejemplo 15/03/2025)." sqref="N5:N58" xr:uid="{90AD2889-AD7E-4F90-9147-892F2A933285}">
+      <formula1>AND(ISNUMBER(N5),N5&gt;=36526)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Fecha invalida" error="Ingrese una fecha valida (por ejemplo 15/03/2025)." sqref="P5:P58" xr:uid="{92A6CE1B-2893-4CA5-A5AC-2C7D963078AF}">
+      <formula1>AND(ISNUMBER(P5),P5&gt;=36526)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9979,64 +10184,64 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="250"/>
-      <c r="B1" s="250"/>
-      <c r="C1" s="250"/>
-      <c r="D1" s="250"/>
-      <c r="E1" s="259" t="s">
+      <c r="A1" s="288"/>
+      <c r="B1" s="288"/>
+      <c r="C1" s="288"/>
+      <c r="D1" s="288"/>
+      <c r="E1" s="292" t="s">
         <v>184</v>
       </c>
-      <c r="F1" s="259"/>
-      <c r="G1" s="259"/>
-      <c r="H1" s="259"/>
-      <c r="I1" s="259"/>
-      <c r="J1" s="259"/>
-      <c r="K1" s="259"/>
-      <c r="L1" s="259"/>
-      <c r="M1" s="250"/>
-      <c r="N1" s="250"/>
-      <c r="O1" s="250"/>
-      <c r="P1" s="250"/>
-      <c r="Q1" s="250"/>
-      <c r="R1" s="250"/>
-      <c r="S1" s="250"/>
-      <c r="T1" s="250"/>
-      <c r="U1" s="250"/>
-      <c r="V1" s="250"/>
-      <c r="W1" s="250"/>
+      <c r="F1" s="292"/>
+      <c r="G1" s="292"/>
+      <c r="H1" s="292"/>
+      <c r="I1" s="292"/>
+      <c r="J1" s="292"/>
+      <c r="K1" s="292"/>
+      <c r="L1" s="292"/>
+      <c r="M1" s="288"/>
+      <c r="N1" s="288"/>
+      <c r="O1" s="288"/>
+      <c r="P1" s="288"/>
+      <c r="Q1" s="288"/>
+      <c r="R1" s="288"/>
+      <c r="S1" s="288"/>
+      <c r="T1" s="288"/>
+      <c r="U1" s="288"/>
+      <c r="V1" s="288"/>
+      <c r="W1" s="288"/>
     </row>
     <row r="2" spans="1:23" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="250"/>
-      <c r="B2" s="250"/>
-      <c r="C2" s="250"/>
-      <c r="D2" s="250"/>
-      <c r="E2" s="260" t="s">
+      <c r="A2" s="288"/>
+      <c r="B2" s="288"/>
+      <c r="C2" s="288"/>
+      <c r="D2" s="288"/>
+      <c r="E2" s="293" t="s">
         <v>185</v>
       </c>
-      <c r="F2" s="260"/>
-      <c r="G2" s="260"/>
-      <c r="H2" s="260"/>
-      <c r="I2" s="260"/>
-      <c r="J2" s="260"/>
-      <c r="K2" s="260"/>
-      <c r="L2" s="260"/>
-      <c r="M2" s="250"/>
-      <c r="N2" s="250"/>
-      <c r="O2" s="250"/>
-      <c r="P2" s="250"/>
-      <c r="Q2" s="250"/>
-      <c r="R2" s="250"/>
-      <c r="S2" s="250"/>
-      <c r="T2" s="250"/>
-      <c r="U2" s="250"/>
-      <c r="V2" s="250"/>
-      <c r="W2" s="250"/>
+      <c r="F2" s="293"/>
+      <c r="G2" s="293"/>
+      <c r="H2" s="293"/>
+      <c r="I2" s="293"/>
+      <c r="J2" s="293"/>
+      <c r="K2" s="293"/>
+      <c r="L2" s="293"/>
+      <c r="M2" s="288"/>
+      <c r="N2" s="288"/>
+      <c r="O2" s="288"/>
+      <c r="P2" s="288"/>
+      <c r="Q2" s="288"/>
+      <c r="R2" s="288"/>
+      <c r="S2" s="288"/>
+      <c r="T2" s="288"/>
+      <c r="U2" s="288"/>
+      <c r="V2" s="288"/>
+      <c r="W2" s="288"/>
     </row>
     <row r="3" spans="1:23" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="250"/>
-      <c r="B3" s="250"/>
-      <c r="C3" s="250"/>
-      <c r="D3" s="250"/>
+      <c r="A3" s="288"/>
+      <c r="B3" s="288"/>
+      <c r="C3" s="288"/>
+      <c r="D3" s="288"/>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
@@ -10045,702 +10250,696 @@
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
-      <c r="M3" s="250"/>
-      <c r="N3" s="250"/>
-      <c r="O3" s="250"/>
-      <c r="P3" s="250"/>
-      <c r="Q3" s="250"/>
-      <c r="R3" s="250"/>
-      <c r="S3" s="250"/>
-      <c r="T3" s="250"/>
-      <c r="U3" s="250"/>
-      <c r="V3" s="250"/>
-      <c r="W3" s="250"/>
+      <c r="M3" s="288"/>
+      <c r="N3" s="288"/>
+      <c r="O3" s="288"/>
+      <c r="P3" s="288"/>
+      <c r="Q3" s="288"/>
+      <c r="R3" s="288"/>
+      <c r="S3" s="288"/>
+      <c r="T3" s="288"/>
+      <c r="U3" s="288"/>
+      <c r="V3" s="288"/>
+      <c r="W3" s="288"/>
     </row>
     <row r="4" spans="1:23" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="250"/>
-      <c r="B4" s="250"/>
-      <c r="C4" s="250"/>
-      <c r="D4" s="250"/>
-      <c r="E4" s="251"/>
-      <c r="F4" s="252"/>
-      <c r="G4" s="252"/>
-      <c r="H4" s="252"/>
-      <c r="I4" s="252"/>
-      <c r="J4" s="252"/>
-      <c r="K4" s="252"/>
-      <c r="L4" s="252"/>
-      <c r="M4" s="250"/>
-      <c r="N4" s="250"/>
-      <c r="O4" s="250"/>
-      <c r="P4" s="250"/>
-      <c r="Q4" s="250"/>
-      <c r="R4" s="250"/>
-      <c r="S4" s="250"/>
-      <c r="T4" s="250"/>
-      <c r="U4" s="250"/>
-      <c r="V4" s="250"/>
-      <c r="W4" s="250"/>
+      <c r="A4" s="288"/>
+      <c r="B4" s="288"/>
+      <c r="C4" s="288"/>
+      <c r="D4" s="288"/>
+      <c r="E4" s="294"/>
+      <c r="F4" s="295"/>
+      <c r="G4" s="295"/>
+      <c r="H4" s="295"/>
+      <c r="I4" s="295"/>
+      <c r="J4" s="295"/>
+      <c r="K4" s="295"/>
+      <c r="L4" s="295"/>
+      <c r="M4" s="288"/>
+      <c r="N4" s="288"/>
+      <c r="O4" s="288"/>
+      <c r="P4" s="288"/>
+      <c r="Q4" s="288"/>
+      <c r="R4" s="288"/>
+      <c r="S4" s="288"/>
+      <c r="T4" s="288"/>
+      <c r="U4" s="288"/>
+      <c r="V4" s="288"/>
+      <c r="W4" s="288"/>
     </row>
     <row r="5" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="250"/>
-      <c r="B5" s="250"/>
-      <c r="C5" s="250"/>
-      <c r="D5" s="250"/>
-      <c r="E5" s="252"/>
-      <c r="F5" s="252"/>
-      <c r="G5" s="252"/>
-      <c r="H5" s="252"/>
-      <c r="I5" s="252"/>
-      <c r="J5" s="252"/>
-      <c r="K5" s="252"/>
-      <c r="L5" s="252"/>
-      <c r="M5" s="250"/>
-      <c r="N5" s="250"/>
-      <c r="O5" s="250"/>
-      <c r="P5" s="250"/>
-      <c r="Q5" s="250"/>
-      <c r="R5" s="250"/>
-      <c r="S5" s="250"/>
-      <c r="T5" s="250"/>
-      <c r="U5" s="250"/>
-      <c r="V5" s="250"/>
-      <c r="W5" s="250"/>
+      <c r="A5" s="288"/>
+      <c r="B5" s="288"/>
+      <c r="C5" s="288"/>
+      <c r="D5" s="288"/>
+      <c r="E5" s="295"/>
+      <c r="F5" s="295"/>
+      <c r="G5" s="295"/>
+      <c r="H5" s="295"/>
+      <c r="I5" s="295"/>
+      <c r="J5" s="295"/>
+      <c r="K5" s="295"/>
+      <c r="L5" s="295"/>
+      <c r="M5" s="288"/>
+      <c r="N5" s="288"/>
+      <c r="O5" s="288"/>
+      <c r="P5" s="288"/>
+      <c r="Q5" s="288"/>
+      <c r="R5" s="288"/>
+      <c r="S5" s="288"/>
+      <c r="T5" s="288"/>
+      <c r="U5" s="288"/>
+      <c r="V5" s="288"/>
+      <c r="W5" s="288"/>
     </row>
     <row r="6" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="250"/>
-      <c r="B6" s="250"/>
-      <c r="C6" s="250"/>
-      <c r="D6" s="250"/>
-      <c r="E6" s="252"/>
-      <c r="F6" s="252"/>
-      <c r="G6" s="252"/>
-      <c r="H6" s="252"/>
-      <c r="I6" s="252"/>
-      <c r="J6" s="252"/>
-      <c r="K6" s="252"/>
-      <c r="L6" s="252"/>
-      <c r="M6" s="250"/>
-      <c r="N6" s="250"/>
-      <c r="O6" s="250"/>
-      <c r="P6" s="250"/>
-      <c r="Q6" s="250"/>
-      <c r="R6" s="250"/>
-      <c r="S6" s="250"/>
-      <c r="T6" s="250"/>
-      <c r="U6" s="250"/>
-      <c r="V6" s="250"/>
-      <c r="W6" s="250"/>
+      <c r="A6" s="288"/>
+      <c r="B6" s="288"/>
+      <c r="C6" s="288"/>
+      <c r="D6" s="288"/>
+      <c r="E6" s="295"/>
+      <c r="F6" s="295"/>
+      <c r="G6" s="295"/>
+      <c r="H6" s="295"/>
+      <c r="I6" s="295"/>
+      <c r="J6" s="295"/>
+      <c r="K6" s="295"/>
+      <c r="L6" s="295"/>
+      <c r="M6" s="288"/>
+      <c r="N6" s="288"/>
+      <c r="O6" s="288"/>
+      <c r="P6" s="288"/>
+      <c r="Q6" s="288"/>
+      <c r="R6" s="288"/>
+      <c r="S6" s="288"/>
+      <c r="T6" s="288"/>
+      <c r="U6" s="288"/>
+      <c r="V6" s="288"/>
+      <c r="W6" s="288"/>
     </row>
     <row r="7" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="250"/>
-      <c r="B7" s="250"/>
-      <c r="C7" s="250"/>
-      <c r="D7" s="250"/>
-      <c r="E7" s="252"/>
-      <c r="F7" s="252"/>
-      <c r="G7" s="252"/>
-      <c r="H7" s="252"/>
-      <c r="I7" s="252"/>
-      <c r="J7" s="252"/>
-      <c r="K7" s="252"/>
-      <c r="L7" s="252"/>
-      <c r="M7" s="250"/>
-      <c r="N7" s="250"/>
-      <c r="O7" s="250"/>
-      <c r="P7" s="250"/>
-      <c r="Q7" s="250"/>
-      <c r="R7" s="250"/>
-      <c r="S7" s="250"/>
-      <c r="T7" s="250"/>
-      <c r="U7" s="250"/>
-      <c r="V7" s="250"/>
-      <c r="W7" s="250"/>
+      <c r="A7" s="288"/>
+      <c r="B7" s="288"/>
+      <c r="C7" s="288"/>
+      <c r="D7" s="288"/>
+      <c r="E7" s="295"/>
+      <c r="F7" s="295"/>
+      <c r="G7" s="295"/>
+      <c r="H7" s="295"/>
+      <c r="I7" s="295"/>
+      <c r="J7" s="295"/>
+      <c r="K7" s="295"/>
+      <c r="L7" s="295"/>
+      <c r="M7" s="288"/>
+      <c r="N7" s="288"/>
+      <c r="O7" s="288"/>
+      <c r="P7" s="288"/>
+      <c r="Q7" s="288"/>
+      <c r="R7" s="288"/>
+      <c r="S7" s="288"/>
+      <c r="T7" s="288"/>
+      <c r="U7" s="288"/>
+      <c r="V7" s="288"/>
+      <c r="W7" s="288"/>
     </row>
     <row r="8" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="250"/>
-      <c r="B8" s="250"/>
-      <c r="C8" s="250"/>
-      <c r="D8" s="250"/>
-      <c r="E8" s="252"/>
-      <c r="F8" s="252"/>
-      <c r="G8" s="252"/>
-      <c r="H8" s="252"/>
-      <c r="I8" s="252"/>
-      <c r="J8" s="252"/>
-      <c r="K8" s="252"/>
-      <c r="L8" s="252"/>
-      <c r="M8" s="250"/>
-      <c r="N8" s="250"/>
-      <c r="O8" s="250"/>
-      <c r="P8" s="250"/>
-      <c r="Q8" s="250"/>
-      <c r="R8" s="250"/>
-      <c r="S8" s="250"/>
-      <c r="T8" s="250"/>
-      <c r="U8" s="250"/>
-      <c r="V8" s="250"/>
-      <c r="W8" s="250"/>
+      <c r="A8" s="288"/>
+      <c r="B8" s="288"/>
+      <c r="C8" s="288"/>
+      <c r="D8" s="288"/>
+      <c r="E8" s="295"/>
+      <c r="F8" s="295"/>
+      <c r="G8" s="295"/>
+      <c r="H8" s="295"/>
+      <c r="I8" s="295"/>
+      <c r="J8" s="295"/>
+      <c r="K8" s="295"/>
+      <c r="L8" s="295"/>
+      <c r="M8" s="288"/>
+      <c r="N8" s="288"/>
+      <c r="O8" s="288"/>
+      <c r="P8" s="288"/>
+      <c r="Q8" s="288"/>
+      <c r="R8" s="288"/>
+      <c r="S8" s="288"/>
+      <c r="T8" s="288"/>
+      <c r="U8" s="288"/>
+      <c r="V8" s="288"/>
+      <c r="W8" s="288"/>
     </row>
     <row r="9" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="250"/>
-      <c r="B9" s="250"/>
-      <c r="C9" s="250"/>
-      <c r="D9" s="250"/>
-      <c r="E9" s="252"/>
-      <c r="F9" s="252"/>
-      <c r="G9" s="252"/>
-      <c r="H9" s="252"/>
-      <c r="I9" s="252"/>
-      <c r="J9" s="252"/>
-      <c r="K9" s="252"/>
-      <c r="L9" s="252"/>
-      <c r="M9" s="250"/>
-      <c r="N9" s="250"/>
-      <c r="O9" s="250"/>
-      <c r="P9" s="250"/>
-      <c r="Q9" s="250"/>
-      <c r="R9" s="250"/>
-      <c r="S9" s="250"/>
-      <c r="T9" s="250"/>
-      <c r="U9" s="250"/>
-      <c r="V9" s="250"/>
-      <c r="W9" s="250"/>
+      <c r="A9" s="288"/>
+      <c r="B9" s="288"/>
+      <c r="C9" s="288"/>
+      <c r="D9" s="288"/>
+      <c r="E9" s="295"/>
+      <c r="F9" s="295"/>
+      <c r="G9" s="295"/>
+      <c r="H9" s="295"/>
+      <c r="I9" s="295"/>
+      <c r="J9" s="295"/>
+      <c r="K9" s="295"/>
+      <c r="L9" s="295"/>
+      <c r="M9" s="288"/>
+      <c r="N9" s="288"/>
+      <c r="O9" s="288"/>
+      <c r="P9" s="288"/>
+      <c r="Q9" s="288"/>
+      <c r="R9" s="288"/>
+      <c r="S9" s="288"/>
+      <c r="T9" s="288"/>
+      <c r="U9" s="288"/>
+      <c r="V9" s="288"/>
+      <c r="W9" s="288"/>
     </row>
     <row r="10" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="250"/>
-      <c r="B10" s="250"/>
-      <c r="C10" s="250"/>
-      <c r="D10" s="250"/>
-      <c r="E10" s="252"/>
-      <c r="F10" s="252"/>
-      <c r="G10" s="252"/>
-      <c r="H10" s="252"/>
-      <c r="I10" s="252"/>
-      <c r="J10" s="252"/>
-      <c r="K10" s="252"/>
-      <c r="L10" s="252"/>
-      <c r="M10" s="250"/>
-      <c r="N10" s="250"/>
-      <c r="O10" s="250"/>
-      <c r="P10" s="250"/>
-      <c r="Q10" s="250"/>
-      <c r="R10" s="250"/>
-      <c r="S10" s="250"/>
-      <c r="T10" s="250"/>
-      <c r="U10" s="250"/>
-      <c r="V10" s="250"/>
-      <c r="W10" s="250"/>
+      <c r="A10" s="288"/>
+      <c r="B10" s="288"/>
+      <c r="C10" s="288"/>
+      <c r="D10" s="288"/>
+      <c r="E10" s="295"/>
+      <c r="F10" s="295"/>
+      <c r="G10" s="295"/>
+      <c r="H10" s="295"/>
+      <c r="I10" s="295"/>
+      <c r="J10" s="295"/>
+      <c r="K10" s="295"/>
+      <c r="L10" s="295"/>
+      <c r="M10" s="288"/>
+      <c r="N10" s="288"/>
+      <c r="O10" s="288"/>
+      <c r="P10" s="288"/>
+      <c r="Q10" s="288"/>
+      <c r="R10" s="288"/>
+      <c r="S10" s="288"/>
+      <c r="T10" s="288"/>
+      <c r="U10" s="288"/>
+      <c r="V10" s="288"/>
+      <c r="W10" s="288"/>
     </row>
     <row r="11" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="250"/>
-      <c r="B11" s="250"/>
-      <c r="C11" s="250"/>
-      <c r="D11" s="250"/>
-      <c r="E11" s="252"/>
-      <c r="F11" s="252"/>
-      <c r="G11" s="252"/>
-      <c r="H11" s="252"/>
-      <c r="I11" s="252"/>
-      <c r="J11" s="252"/>
-      <c r="K11" s="252"/>
-      <c r="L11" s="252"/>
-      <c r="M11" s="250"/>
-      <c r="N11" s="250"/>
-      <c r="O11" s="250"/>
-      <c r="P11" s="250"/>
-      <c r="Q11" s="250"/>
-      <c r="R11" s="250"/>
-      <c r="S11" s="250"/>
-      <c r="T11" s="250"/>
-      <c r="U11" s="250"/>
-      <c r="V11" s="250"/>
-      <c r="W11" s="250"/>
+      <c r="A11" s="288"/>
+      <c r="B11" s="288"/>
+      <c r="C11" s="288"/>
+      <c r="D11" s="288"/>
+      <c r="E11" s="295"/>
+      <c r="F11" s="295"/>
+      <c r="G11" s="295"/>
+      <c r="H11" s="295"/>
+      <c r="I11" s="295"/>
+      <c r="J11" s="295"/>
+      <c r="K11" s="295"/>
+      <c r="L11" s="295"/>
+      <c r="M11" s="288"/>
+      <c r="N11" s="288"/>
+      <c r="O11" s="288"/>
+      <c r="P11" s="288"/>
+      <c r="Q11" s="288"/>
+      <c r="R11" s="288"/>
+      <c r="S11" s="288"/>
+      <c r="T11" s="288"/>
+      <c r="U11" s="288"/>
+      <c r="V11" s="288"/>
+      <c r="W11" s="288"/>
     </row>
     <row r="12" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="250"/>
-      <c r="B12" s="250"/>
-      <c r="C12" s="250"/>
-      <c r="D12" s="250"/>
-      <c r="E12" s="252"/>
-      <c r="F12" s="252"/>
-      <c r="G12" s="252"/>
-      <c r="H12" s="252"/>
-      <c r="I12" s="252"/>
-      <c r="J12" s="252"/>
-      <c r="K12" s="252"/>
-      <c r="L12" s="252"/>
-      <c r="M12" s="250"/>
-      <c r="N12" s="250"/>
-      <c r="O12" s="250"/>
-      <c r="P12" s="250"/>
-      <c r="Q12" s="250"/>
-      <c r="R12" s="250"/>
-      <c r="S12" s="250"/>
-      <c r="T12" s="250"/>
-      <c r="U12" s="250"/>
-      <c r="V12" s="250"/>
-      <c r="W12" s="250"/>
+      <c r="A12" s="288"/>
+      <c r="B12" s="288"/>
+      <c r="C12" s="288"/>
+      <c r="D12" s="288"/>
+      <c r="E12" s="295"/>
+      <c r="F12" s="295"/>
+      <c r="G12" s="295"/>
+      <c r="H12" s="295"/>
+      <c r="I12" s="295"/>
+      <c r="J12" s="295"/>
+      <c r="K12" s="295"/>
+      <c r="L12" s="295"/>
+      <c r="M12" s="288"/>
+      <c r="N12" s="288"/>
+      <c r="O12" s="288"/>
+      <c r="P12" s="288"/>
+      <c r="Q12" s="288"/>
+      <c r="R12" s="288"/>
+      <c r="S12" s="288"/>
+      <c r="T12" s="288"/>
+      <c r="U12" s="288"/>
+      <c r="V12" s="288"/>
+      <c r="W12" s="288"/>
     </row>
     <row r="13" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="250"/>
-      <c r="B13" s="250"/>
-      <c r="C13" s="250"/>
-      <c r="D13" s="250"/>
-      <c r="E13" s="252"/>
-      <c r="F13" s="252"/>
-      <c r="G13" s="252"/>
-      <c r="H13" s="252"/>
-      <c r="I13" s="252"/>
-      <c r="J13" s="252"/>
-      <c r="K13" s="252"/>
-      <c r="L13" s="252"/>
-      <c r="M13" s="250"/>
-      <c r="N13" s="250"/>
-      <c r="O13" s="250"/>
-      <c r="P13" s="250"/>
-      <c r="Q13" s="250"/>
-      <c r="R13" s="250"/>
-      <c r="S13" s="250"/>
-      <c r="T13" s="250"/>
-      <c r="U13" s="250"/>
-      <c r="V13" s="250"/>
-      <c r="W13" s="250"/>
+      <c r="A13" s="288"/>
+      <c r="B13" s="288"/>
+      <c r="C13" s="288"/>
+      <c r="D13" s="288"/>
+      <c r="E13" s="295"/>
+      <c r="F13" s="295"/>
+      <c r="G13" s="295"/>
+      <c r="H13" s="295"/>
+      <c r="I13" s="295"/>
+      <c r="J13" s="295"/>
+      <c r="K13" s="295"/>
+      <c r="L13" s="295"/>
+      <c r="M13" s="288"/>
+      <c r="N13" s="288"/>
+      <c r="O13" s="288"/>
+      <c r="P13" s="288"/>
+      <c r="Q13" s="288"/>
+      <c r="R13" s="288"/>
+      <c r="S13" s="288"/>
+      <c r="T13" s="288"/>
+      <c r="U13" s="288"/>
+      <c r="V13" s="288"/>
+      <c r="W13" s="288"/>
     </row>
     <row r="14" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="250"/>
-      <c r="B14" s="250"/>
-      <c r="C14" s="250"/>
-      <c r="D14" s="250"/>
-      <c r="E14" s="252"/>
-      <c r="F14" s="252"/>
-      <c r="G14" s="252"/>
-      <c r="H14" s="252"/>
-      <c r="I14" s="252"/>
-      <c r="J14" s="252"/>
-      <c r="K14" s="252"/>
-      <c r="L14" s="252"/>
-      <c r="M14" s="250"/>
-      <c r="N14" s="250"/>
-      <c r="O14" s="250"/>
-      <c r="P14" s="250"/>
-      <c r="Q14" s="250"/>
-      <c r="R14" s="250"/>
-      <c r="S14" s="250"/>
-      <c r="T14" s="250"/>
-      <c r="U14" s="250"/>
-      <c r="V14" s="250"/>
-      <c r="W14" s="250"/>
+      <c r="A14" s="288"/>
+      <c r="B14" s="288"/>
+      <c r="C14" s="288"/>
+      <c r="D14" s="288"/>
+      <c r="E14" s="295"/>
+      <c r="F14" s="295"/>
+      <c r="G14" s="295"/>
+      <c r="H14" s="295"/>
+      <c r="I14" s="295"/>
+      <c r="J14" s="295"/>
+      <c r="K14" s="295"/>
+      <c r="L14" s="295"/>
+      <c r="M14" s="288"/>
+      <c r="N14" s="288"/>
+      <c r="O14" s="288"/>
+      <c r="P14" s="288"/>
+      <c r="Q14" s="288"/>
+      <c r="R14" s="288"/>
+      <c r="S14" s="288"/>
+      <c r="T14" s="288"/>
+      <c r="U14" s="288"/>
+      <c r="V14" s="288"/>
+      <c r="W14" s="288"/>
     </row>
     <row r="15" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="250"/>
-      <c r="B15" s="250"/>
-      <c r="C15" s="250"/>
-      <c r="D15" s="250"/>
-      <c r="E15" s="252"/>
-      <c r="F15" s="252"/>
-      <c r="G15" s="252"/>
-      <c r="H15" s="252"/>
-      <c r="I15" s="252"/>
-      <c r="J15" s="252"/>
-      <c r="K15" s="252"/>
-      <c r="L15" s="252"/>
-      <c r="M15" s="250"/>
-      <c r="N15" s="250"/>
-      <c r="O15" s="250"/>
-      <c r="P15" s="250"/>
-      <c r="Q15" s="250"/>
-      <c r="R15" s="250"/>
-      <c r="S15" s="250"/>
-      <c r="T15" s="250"/>
-      <c r="U15" s="250"/>
-      <c r="V15" s="250"/>
-      <c r="W15" s="250"/>
+      <c r="A15" s="288"/>
+      <c r="B15" s="288"/>
+      <c r="C15" s="288"/>
+      <c r="D15" s="288"/>
+      <c r="E15" s="295"/>
+      <c r="F15" s="295"/>
+      <c r="G15" s="295"/>
+      <c r="H15" s="295"/>
+      <c r="I15" s="295"/>
+      <c r="J15" s="295"/>
+      <c r="K15" s="295"/>
+      <c r="L15" s="295"/>
+      <c r="M15" s="288"/>
+      <c r="N15" s="288"/>
+      <c r="O15" s="288"/>
+      <c r="P15" s="288"/>
+      <c r="Q15" s="288"/>
+      <c r="R15" s="288"/>
+      <c r="S15" s="288"/>
+      <c r="T15" s="288"/>
+      <c r="U15" s="288"/>
+      <c r="V15" s="288"/>
+      <c r="W15" s="288"/>
     </row>
     <row r="16" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="250"/>
-      <c r="B16" s="250"/>
-      <c r="C16" s="250"/>
-      <c r="D16" s="250"/>
-      <c r="E16" s="252"/>
-      <c r="F16" s="252"/>
-      <c r="G16" s="252"/>
-      <c r="H16" s="252"/>
-      <c r="I16" s="252"/>
-      <c r="J16" s="252"/>
-      <c r="K16" s="252"/>
-      <c r="L16" s="252"/>
-      <c r="M16" s="250"/>
-      <c r="N16" s="250"/>
-      <c r="O16" s="250"/>
-      <c r="P16" s="250"/>
-      <c r="Q16" s="250"/>
-      <c r="R16" s="250"/>
-      <c r="S16" s="250"/>
-      <c r="T16" s="250"/>
-      <c r="U16" s="250"/>
-      <c r="V16" s="250"/>
-      <c r="W16" s="250"/>
+      <c r="A16" s="288"/>
+      <c r="B16" s="288"/>
+      <c r="C16" s="288"/>
+      <c r="D16" s="288"/>
+      <c r="E16" s="295"/>
+      <c r="F16" s="295"/>
+      <c r="G16" s="295"/>
+      <c r="H16" s="295"/>
+      <c r="I16" s="295"/>
+      <c r="J16" s="295"/>
+      <c r="K16" s="295"/>
+      <c r="L16" s="295"/>
+      <c r="M16" s="288"/>
+      <c r="N16" s="288"/>
+      <c r="O16" s="288"/>
+      <c r="P16" s="288"/>
+      <c r="Q16" s="288"/>
+      <c r="R16" s="288"/>
+      <c r="S16" s="288"/>
+      <c r="T16" s="288"/>
+      <c r="U16" s="288"/>
+      <c r="V16" s="288"/>
+      <c r="W16" s="288"/>
     </row>
     <row r="17" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="250"/>
-      <c r="B17" s="250"/>
-      <c r="C17" s="250"/>
-      <c r="D17" s="250"/>
-      <c r="E17" s="252"/>
-      <c r="F17" s="252"/>
-      <c r="G17" s="252"/>
-      <c r="H17" s="252"/>
-      <c r="I17" s="252"/>
-      <c r="J17" s="252"/>
-      <c r="K17" s="252"/>
-      <c r="L17" s="252"/>
-      <c r="M17" s="250"/>
-      <c r="N17" s="250"/>
-      <c r="O17" s="250"/>
-      <c r="P17" s="250"/>
-      <c r="Q17" s="250"/>
-      <c r="R17" s="250"/>
-      <c r="S17" s="250"/>
-      <c r="T17" s="250"/>
-      <c r="U17" s="250"/>
-      <c r="V17" s="250"/>
-      <c r="W17" s="250"/>
+      <c r="A17" s="288"/>
+      <c r="B17" s="288"/>
+      <c r="C17" s="288"/>
+      <c r="D17" s="288"/>
+      <c r="E17" s="295"/>
+      <c r="F17" s="295"/>
+      <c r="G17" s="295"/>
+      <c r="H17" s="295"/>
+      <c r="I17" s="295"/>
+      <c r="J17" s="295"/>
+      <c r="K17" s="295"/>
+      <c r="L17" s="295"/>
+      <c r="M17" s="288"/>
+      <c r="N17" s="288"/>
+      <c r="O17" s="288"/>
+      <c r="P17" s="288"/>
+      <c r="Q17" s="288"/>
+      <c r="R17" s="288"/>
+      <c r="S17" s="288"/>
+      <c r="T17" s="288"/>
+      <c r="U17" s="288"/>
+      <c r="V17" s="288"/>
+      <c r="W17" s="288"/>
     </row>
     <row r="18" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="250"/>
-      <c r="B18" s="250"/>
-      <c r="C18" s="250"/>
-      <c r="D18" s="250"/>
-      <c r="E18" s="252"/>
-      <c r="F18" s="252"/>
-      <c r="G18" s="252"/>
-      <c r="H18" s="252"/>
-      <c r="I18" s="252"/>
-      <c r="J18" s="252"/>
-      <c r="K18" s="252"/>
-      <c r="L18" s="252"/>
-      <c r="M18" s="250"/>
-      <c r="N18" s="250"/>
-      <c r="O18" s="250"/>
-      <c r="P18" s="250"/>
-      <c r="Q18" s="250"/>
-      <c r="R18" s="250"/>
-      <c r="S18" s="250"/>
-      <c r="T18" s="250"/>
-      <c r="U18" s="250"/>
-      <c r="V18" s="250"/>
-      <c r="W18" s="250"/>
+      <c r="A18" s="288"/>
+      <c r="B18" s="288"/>
+      <c r="C18" s="288"/>
+      <c r="D18" s="288"/>
+      <c r="E18" s="295"/>
+      <c r="F18" s="295"/>
+      <c r="G18" s="295"/>
+      <c r="H18" s="295"/>
+      <c r="I18" s="295"/>
+      <c r="J18" s="295"/>
+      <c r="K18" s="295"/>
+      <c r="L18" s="295"/>
+      <c r="M18" s="288"/>
+      <c r="N18" s="288"/>
+      <c r="O18" s="288"/>
+      <c r="P18" s="288"/>
+      <c r="Q18" s="288"/>
+      <c r="R18" s="288"/>
+      <c r="S18" s="288"/>
+      <c r="T18" s="288"/>
+      <c r="U18" s="288"/>
+      <c r="V18" s="288"/>
+      <c r="W18" s="288"/>
     </row>
     <row r="19" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="250"/>
-      <c r="B19" s="250"/>
-      <c r="C19" s="250"/>
-      <c r="D19" s="250"/>
-      <c r="E19" s="252"/>
-      <c r="F19" s="252"/>
-      <c r="G19" s="252"/>
-      <c r="H19" s="252"/>
-      <c r="I19" s="252"/>
-      <c r="J19" s="252"/>
-      <c r="K19" s="252"/>
-      <c r="L19" s="252"/>
-      <c r="M19" s="250"/>
-      <c r="N19" s="250"/>
-      <c r="O19" s="250"/>
-      <c r="P19" s="250"/>
-      <c r="Q19" s="250"/>
-      <c r="R19" s="250"/>
-      <c r="S19" s="250"/>
-      <c r="T19" s="250"/>
-      <c r="U19" s="250"/>
-      <c r="V19" s="250"/>
-      <c r="W19" s="250"/>
+      <c r="A19" s="288"/>
+      <c r="B19" s="288"/>
+      <c r="C19" s="288"/>
+      <c r="D19" s="288"/>
+      <c r="E19" s="295"/>
+      <c r="F19" s="295"/>
+      <c r="G19" s="295"/>
+      <c r="H19" s="295"/>
+      <c r="I19" s="295"/>
+      <c r="J19" s="295"/>
+      <c r="K19" s="295"/>
+      <c r="L19" s="295"/>
+      <c r="M19" s="288"/>
+      <c r="N19" s="288"/>
+      <c r="O19" s="288"/>
+      <c r="P19" s="288"/>
+      <c r="Q19" s="288"/>
+      <c r="R19" s="288"/>
+      <c r="S19" s="288"/>
+      <c r="T19" s="288"/>
+      <c r="U19" s="288"/>
+      <c r="V19" s="288"/>
+      <c r="W19" s="288"/>
     </row>
     <row r="20" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="250"/>
-      <c r="B20" s="250"/>
-      <c r="C20" s="250"/>
-      <c r="D20" s="250"/>
-      <c r="E20" s="252"/>
-      <c r="F20" s="252"/>
-      <c r="G20" s="252"/>
-      <c r="H20" s="252"/>
-      <c r="I20" s="252"/>
-      <c r="J20" s="252"/>
-      <c r="K20" s="252"/>
-      <c r="L20" s="252"/>
-      <c r="M20" s="250"/>
-      <c r="N20" s="250"/>
-      <c r="O20" s="250"/>
-      <c r="P20" s="250"/>
-      <c r="Q20" s="250"/>
-      <c r="R20" s="250"/>
-      <c r="S20" s="250"/>
-      <c r="T20" s="250"/>
-      <c r="U20" s="250"/>
-      <c r="V20" s="250"/>
-      <c r="W20" s="250"/>
+      <c r="A20" s="288"/>
+      <c r="B20" s="288"/>
+      <c r="C20" s="288"/>
+      <c r="D20" s="288"/>
+      <c r="E20" s="295"/>
+      <c r="F20" s="295"/>
+      <c r="G20" s="295"/>
+      <c r="H20" s="295"/>
+      <c r="I20" s="295"/>
+      <c r="J20" s="295"/>
+      <c r="K20" s="295"/>
+      <c r="L20" s="295"/>
+      <c r="M20" s="288"/>
+      <c r="N20" s="288"/>
+      <c r="O20" s="288"/>
+      <c r="P20" s="288"/>
+      <c r="Q20" s="288"/>
+      <c r="R20" s="288"/>
+      <c r="S20" s="288"/>
+      <c r="T20" s="288"/>
+      <c r="U20" s="288"/>
+      <c r="V20" s="288"/>
+      <c r="W20" s="288"/>
     </row>
     <row r="21" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="250"/>
-      <c r="B21" s="250"/>
-      <c r="C21" s="250"/>
-      <c r="D21" s="250"/>
-      <c r="E21" s="252"/>
-      <c r="F21" s="252"/>
-      <c r="G21" s="252"/>
-      <c r="H21" s="252"/>
-      <c r="I21" s="252"/>
-      <c r="J21" s="252"/>
-      <c r="K21" s="252"/>
-      <c r="L21" s="252"/>
-      <c r="M21" s="250"/>
-      <c r="N21" s="250"/>
-      <c r="O21" s="250"/>
-      <c r="P21" s="250"/>
-      <c r="Q21" s="250"/>
-      <c r="R21" s="250"/>
-      <c r="S21" s="250"/>
-      <c r="T21" s="250"/>
-      <c r="U21" s="250"/>
-      <c r="V21" s="250"/>
-      <c r="W21" s="250"/>
+      <c r="A21" s="288"/>
+      <c r="B21" s="288"/>
+      <c r="C21" s="288"/>
+      <c r="D21" s="288"/>
+      <c r="E21" s="295"/>
+      <c r="F21" s="295"/>
+      <c r="G21" s="295"/>
+      <c r="H21" s="295"/>
+      <c r="I21" s="295"/>
+      <c r="J21" s="295"/>
+      <c r="K21" s="295"/>
+      <c r="L21" s="295"/>
+      <c r="M21" s="288"/>
+      <c r="N21" s="288"/>
+      <c r="O21" s="288"/>
+      <c r="P21" s="288"/>
+      <c r="Q21" s="288"/>
+      <c r="R21" s="288"/>
+      <c r="S21" s="288"/>
+      <c r="T21" s="288"/>
+      <c r="U21" s="288"/>
+      <c r="V21" s="288"/>
+      <c r="W21" s="288"/>
     </row>
     <row r="22" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="250"/>
-      <c r="B22" s="250"/>
-      <c r="C22" s="250"/>
-      <c r="D22" s="250"/>
-      <c r="E22" s="252"/>
-      <c r="F22" s="252"/>
-      <c r="G22" s="252"/>
-      <c r="H22" s="252"/>
-      <c r="I22" s="252"/>
-      <c r="J22" s="252"/>
-      <c r="K22" s="252"/>
-      <c r="L22" s="252"/>
-      <c r="M22" s="250"/>
-      <c r="N22" s="250"/>
-      <c r="O22" s="250"/>
-      <c r="P22" s="250"/>
-      <c r="Q22" s="250"/>
-      <c r="R22" s="250"/>
-      <c r="S22" s="250"/>
-      <c r="T22" s="250"/>
-      <c r="U22" s="250"/>
-      <c r="V22" s="250"/>
-      <c r="W22" s="250"/>
+      <c r="A22" s="288"/>
+      <c r="B22" s="288"/>
+      <c r="C22" s="288"/>
+      <c r="D22" s="288"/>
+      <c r="E22" s="295"/>
+      <c r="F22" s="295"/>
+      <c r="G22" s="295"/>
+      <c r="H22" s="295"/>
+      <c r="I22" s="295"/>
+      <c r="J22" s="295"/>
+      <c r="K22" s="295"/>
+      <c r="L22" s="295"/>
+      <c r="M22" s="288"/>
+      <c r="N22" s="288"/>
+      <c r="O22" s="288"/>
+      <c r="P22" s="288"/>
+      <c r="Q22" s="288"/>
+      <c r="R22" s="288"/>
+      <c r="S22" s="288"/>
+      <c r="T22" s="288"/>
+      <c r="U22" s="288"/>
+      <c r="V22" s="288"/>
+      <c r="W22" s="288"/>
     </row>
     <row r="23" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="250"/>
-      <c r="B23" s="250"/>
-      <c r="C23" s="250"/>
-      <c r="D23" s="250"/>
-      <c r="E23" s="253"/>
-      <c r="F23" s="254"/>
-      <c r="G23" s="254"/>
-      <c r="H23" s="254"/>
-      <c r="I23" s="254"/>
-      <c r="J23" s="254"/>
-      <c r="K23" s="254"/>
-      <c r="L23" s="255"/>
-      <c r="M23" s="250"/>
-      <c r="N23" s="250"/>
-      <c r="O23" s="250"/>
-      <c r="P23" s="250"/>
-      <c r="Q23" s="250"/>
-      <c r="R23" s="250"/>
-      <c r="S23" s="250"/>
-      <c r="T23" s="250"/>
-      <c r="U23" s="250"/>
-      <c r="V23" s="250"/>
-      <c r="W23" s="250"/>
+      <c r="A23" s="288"/>
+      <c r="B23" s="288"/>
+      <c r="C23" s="288"/>
+      <c r="D23" s="288"/>
+      <c r="E23" s="289"/>
+      <c r="F23" s="290"/>
+      <c r="G23" s="290"/>
+      <c r="H23" s="290"/>
+      <c r="I23" s="290"/>
+      <c r="J23" s="290"/>
+      <c r="K23" s="290"/>
+      <c r="L23" s="291"/>
+      <c r="M23" s="288"/>
+      <c r="N23" s="288"/>
+      <c r="O23" s="288"/>
+      <c r="P23" s="288"/>
+      <c r="Q23" s="288"/>
+      <c r="R23" s="288"/>
+      <c r="S23" s="288"/>
+      <c r="T23" s="288"/>
+      <c r="U23" s="288"/>
+      <c r="V23" s="288"/>
+      <c r="W23" s="288"/>
     </row>
     <row r="24" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="250"/>
-      <c r="B24" s="250"/>
-      <c r="C24" s="250"/>
-      <c r="D24" s="250"/>
-      <c r="E24" s="253"/>
-      <c r="F24" s="254"/>
-      <c r="G24" s="254"/>
-      <c r="H24" s="254"/>
-      <c r="I24" s="254"/>
-      <c r="J24" s="254"/>
-      <c r="K24" s="254"/>
-      <c r="L24" s="255"/>
-      <c r="M24" s="250"/>
-      <c r="N24" s="250"/>
-      <c r="O24" s="250"/>
-      <c r="P24" s="250"/>
-      <c r="Q24" s="250"/>
-      <c r="R24" s="250"/>
-      <c r="S24" s="250"/>
-      <c r="T24" s="250"/>
-      <c r="U24" s="250"/>
-      <c r="V24" s="250"/>
-      <c r="W24" s="250"/>
+      <c r="A24" s="288"/>
+      <c r="B24" s="288"/>
+      <c r="C24" s="288"/>
+      <c r="D24" s="288"/>
+      <c r="E24" s="289"/>
+      <c r="F24" s="290"/>
+      <c r="G24" s="290"/>
+      <c r="H24" s="290"/>
+      <c r="I24" s="290"/>
+      <c r="J24" s="290"/>
+      <c r="K24" s="290"/>
+      <c r="L24" s="291"/>
+      <c r="M24" s="288"/>
+      <c r="N24" s="288"/>
+      <c r="O24" s="288"/>
+      <c r="P24" s="288"/>
+      <c r="Q24" s="288"/>
+      <c r="R24" s="288"/>
+      <c r="S24" s="288"/>
+      <c r="T24" s="288"/>
+      <c r="U24" s="288"/>
+      <c r="V24" s="288"/>
+      <c r="W24" s="288"/>
     </row>
     <row r="25" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="250"/>
-      <c r="B25" s="250"/>
-      <c r="C25" s="250"/>
-      <c r="D25" s="250"/>
-      <c r="E25" s="253"/>
-      <c r="F25" s="254"/>
-      <c r="G25" s="254"/>
-      <c r="H25" s="254"/>
-      <c r="I25" s="254"/>
-      <c r="J25" s="254"/>
-      <c r="K25" s="254"/>
-      <c r="L25" s="255"/>
-      <c r="M25" s="250"/>
-      <c r="N25" s="250"/>
-      <c r="O25" s="250"/>
-      <c r="P25" s="250"/>
-      <c r="Q25" s="250"/>
-      <c r="R25" s="250"/>
-      <c r="S25" s="250"/>
-      <c r="T25" s="250"/>
-      <c r="U25" s="250"/>
-      <c r="V25" s="250"/>
-      <c r="W25" s="250"/>
+      <c r="A25" s="288"/>
+      <c r="B25" s="288"/>
+      <c r="C25" s="288"/>
+      <c r="D25" s="288"/>
+      <c r="E25" s="289"/>
+      <c r="F25" s="290"/>
+      <c r="G25" s="290"/>
+      <c r="H25" s="290"/>
+      <c r="I25" s="290"/>
+      <c r="J25" s="290"/>
+      <c r="K25" s="290"/>
+      <c r="L25" s="291"/>
+      <c r="M25" s="288"/>
+      <c r="N25" s="288"/>
+      <c r="O25" s="288"/>
+      <c r="P25" s="288"/>
+      <c r="Q25" s="288"/>
+      <c r="R25" s="288"/>
+      <c r="S25" s="288"/>
+      <c r="T25" s="288"/>
+      <c r="U25" s="288"/>
+      <c r="V25" s="288"/>
+      <c r="W25" s="288"/>
     </row>
     <row r="26" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="250"/>
-      <c r="B26" s="250"/>
-      <c r="C26" s="250"/>
-      <c r="D26" s="250"/>
-      <c r="E26" s="253"/>
-      <c r="F26" s="254"/>
-      <c r="G26" s="254"/>
-      <c r="H26" s="254"/>
-      <c r="I26" s="254"/>
-      <c r="J26" s="254"/>
-      <c r="K26" s="254"/>
-      <c r="L26" s="255"/>
-      <c r="M26" s="250"/>
-      <c r="N26" s="250"/>
-      <c r="O26" s="250"/>
-      <c r="P26" s="250"/>
-      <c r="Q26" s="250"/>
-      <c r="R26" s="250"/>
-      <c r="S26" s="250"/>
-      <c r="T26" s="250"/>
-      <c r="U26" s="250"/>
-      <c r="V26" s="250"/>
-      <c r="W26" s="250"/>
+      <c r="A26" s="288"/>
+      <c r="B26" s="288"/>
+      <c r="C26" s="288"/>
+      <c r="D26" s="288"/>
+      <c r="E26" s="289"/>
+      <c r="F26" s="290"/>
+      <c r="G26" s="290"/>
+      <c r="H26" s="290"/>
+      <c r="I26" s="290"/>
+      <c r="J26" s="290"/>
+      <c r="K26" s="290"/>
+      <c r="L26" s="291"/>
+      <c r="M26" s="288"/>
+      <c r="N26" s="288"/>
+      <c r="O26" s="288"/>
+      <c r="P26" s="288"/>
+      <c r="Q26" s="288"/>
+      <c r="R26" s="288"/>
+      <c r="S26" s="288"/>
+      <c r="T26" s="288"/>
+      <c r="U26" s="288"/>
+      <c r="V26" s="288"/>
+      <c r="W26" s="288"/>
     </row>
     <row r="27" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="250"/>
-      <c r="B27" s="250"/>
-      <c r="C27" s="250"/>
-      <c r="D27" s="250"/>
-      <c r="E27" s="253"/>
-      <c r="F27" s="254"/>
-      <c r="G27" s="254"/>
-      <c r="H27" s="254"/>
-      <c r="I27" s="254"/>
-      <c r="J27" s="254"/>
-      <c r="K27" s="254"/>
-      <c r="L27" s="255"/>
-      <c r="M27" s="250"/>
-      <c r="N27" s="250"/>
-      <c r="O27" s="250"/>
-      <c r="P27" s="250"/>
-      <c r="Q27" s="250"/>
-      <c r="R27" s="250"/>
-      <c r="S27" s="250"/>
-      <c r="T27" s="250"/>
-      <c r="U27" s="250"/>
-      <c r="V27" s="250"/>
-      <c r="W27" s="250"/>
+      <c r="A27" s="288"/>
+      <c r="B27" s="288"/>
+      <c r="C27" s="288"/>
+      <c r="D27" s="288"/>
+      <c r="E27" s="289"/>
+      <c r="F27" s="290"/>
+      <c r="G27" s="290"/>
+      <c r="H27" s="290"/>
+      <c r="I27" s="290"/>
+      <c r="J27" s="290"/>
+      <c r="K27" s="290"/>
+      <c r="L27" s="291"/>
+      <c r="M27" s="288"/>
+      <c r="N27" s="288"/>
+      <c r="O27" s="288"/>
+      <c r="P27" s="288"/>
+      <c r="Q27" s="288"/>
+      <c r="R27" s="288"/>
+      <c r="S27" s="288"/>
+      <c r="T27" s="288"/>
+      <c r="U27" s="288"/>
+      <c r="V27" s="288"/>
+      <c r="W27" s="288"/>
     </row>
     <row r="28" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="250"/>
-      <c r="B28" s="250"/>
-      <c r="C28" s="250"/>
-      <c r="D28" s="250"/>
-      <c r="E28" s="253"/>
-      <c r="F28" s="254"/>
-      <c r="G28" s="254"/>
-      <c r="H28" s="254"/>
-      <c r="I28" s="254"/>
-      <c r="J28" s="254"/>
-      <c r="K28" s="254"/>
-      <c r="L28" s="255"/>
-      <c r="M28" s="250"/>
-      <c r="N28" s="250"/>
-      <c r="O28" s="250"/>
-      <c r="P28" s="250"/>
-      <c r="Q28" s="250"/>
-      <c r="R28" s="250"/>
-      <c r="S28" s="250"/>
-      <c r="T28" s="250"/>
-      <c r="U28" s="250"/>
-      <c r="V28" s="250"/>
-      <c r="W28" s="250"/>
+      <c r="A28" s="288"/>
+      <c r="B28" s="288"/>
+      <c r="C28" s="288"/>
+      <c r="D28" s="288"/>
+      <c r="E28" s="289"/>
+      <c r="F28" s="290"/>
+      <c r="G28" s="290"/>
+      <c r="H28" s="290"/>
+      <c r="I28" s="290"/>
+      <c r="J28" s="290"/>
+      <c r="K28" s="290"/>
+      <c r="L28" s="291"/>
+      <c r="M28" s="288"/>
+      <c r="N28" s="288"/>
+      <c r="O28" s="288"/>
+      <c r="P28" s="288"/>
+      <c r="Q28" s="288"/>
+      <c r="R28" s="288"/>
+      <c r="S28" s="288"/>
+      <c r="T28" s="288"/>
+      <c r="U28" s="288"/>
+      <c r="V28" s="288"/>
+      <c r="W28" s="288"/>
     </row>
     <row r="29" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="250"/>
-      <c r="B29" s="250"/>
-      <c r="C29" s="250"/>
-      <c r="D29" s="250"/>
-      <c r="E29" s="253"/>
-      <c r="F29" s="254"/>
-      <c r="G29" s="254"/>
-      <c r="H29" s="254"/>
-      <c r="I29" s="254"/>
-      <c r="J29" s="254"/>
-      <c r="K29" s="254"/>
-      <c r="L29" s="255"/>
-      <c r="M29" s="250"/>
-      <c r="N29" s="250"/>
-      <c r="O29" s="250"/>
-      <c r="P29" s="250"/>
-      <c r="Q29" s="250"/>
-      <c r="R29" s="250"/>
-      <c r="S29" s="250"/>
-      <c r="T29" s="250"/>
-      <c r="U29" s="250"/>
-      <c r="V29" s="250"/>
-      <c r="W29" s="250"/>
+      <c r="A29" s="288"/>
+      <c r="B29" s="288"/>
+      <c r="C29" s="288"/>
+      <c r="D29" s="288"/>
+      <c r="E29" s="289"/>
+      <c r="F29" s="290"/>
+      <c r="G29" s="290"/>
+      <c r="H29" s="290"/>
+      <c r="I29" s="290"/>
+      <c r="J29" s="290"/>
+      <c r="K29" s="290"/>
+      <c r="L29" s="291"/>
+      <c r="M29" s="288"/>
+      <c r="N29" s="288"/>
+      <c r="O29" s="288"/>
+      <c r="P29" s="288"/>
+      <c r="Q29" s="288"/>
+      <c r="R29" s="288"/>
+      <c r="S29" s="288"/>
+      <c r="T29" s="288"/>
+      <c r="U29" s="288"/>
+      <c r="V29" s="288"/>
+      <c r="W29" s="288"/>
     </row>
     <row r="30" spans="1:23" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="250"/>
-      <c r="B30" s="250"/>
-      <c r="C30" s="250"/>
-      <c r="D30" s="250"/>
-      <c r="E30" s="256"/>
-      <c r="F30" s="257"/>
-      <c r="G30" s="257"/>
-      <c r="H30" s="257"/>
-      <c r="I30" s="257"/>
-      <c r="J30" s="257"/>
-      <c r="K30" s="257"/>
-      <c r="L30" s="258"/>
-      <c r="M30" s="250"/>
-      <c r="N30" s="250"/>
-      <c r="O30" s="250"/>
-      <c r="P30" s="250"/>
-      <c r="Q30" s="250"/>
-      <c r="R30" s="250"/>
-      <c r="S30" s="250"/>
-      <c r="T30" s="250"/>
-      <c r="U30" s="250"/>
-      <c r="V30" s="250"/>
-      <c r="W30" s="250"/>
+      <c r="A30" s="288"/>
+      <c r="B30" s="288"/>
+      <c r="C30" s="288"/>
+      <c r="D30" s="288"/>
+      <c r="E30" s="296"/>
+      <c r="F30" s="297"/>
+      <c r="G30" s="297"/>
+      <c r="H30" s="297"/>
+      <c r="I30" s="297"/>
+      <c r="J30" s="297"/>
+      <c r="K30" s="297"/>
+      <c r="L30" s="298"/>
+      <c r="M30" s="288"/>
+      <c r="N30" s="288"/>
+      <c r="O30" s="288"/>
+      <c r="P30" s="288"/>
+      <c r="Q30" s="288"/>
+      <c r="R30" s="288"/>
+      <c r="S30" s="288"/>
+      <c r="T30" s="288"/>
+      <c r="U30" s="288"/>
+      <c r="V30" s="288"/>
+      <c r="W30" s="288"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="13">
-    <mergeCell ref="A1:D30"/>
-    <mergeCell ref="E23:L23"/>
-    <mergeCell ref="E24:L24"/>
-    <mergeCell ref="E25:L25"/>
-    <mergeCell ref="E1:L1"/>
-    <mergeCell ref="E2:L2"/>
     <mergeCell ref="M1:W30"/>
     <mergeCell ref="E4:L22"/>
     <mergeCell ref="E26:L26"/>
@@ -10748,6 +10947,12 @@
     <mergeCell ref="E28:L28"/>
     <mergeCell ref="E29:L29"/>
     <mergeCell ref="E30:L30"/>
+    <mergeCell ref="A1:D30"/>
+    <mergeCell ref="E23:L23"/>
+    <mergeCell ref="E24:L24"/>
+    <mergeCell ref="E25:L25"/>
+    <mergeCell ref="E1:L1"/>
+    <mergeCell ref="E2:L2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>